<commit_message>
Record BRT coverage check and freeze search string v0.3
Judged a random sample of 50 of the 298 Scopus records that a broad BRT
query returns but v0.3 misses: 0 relevant, 0 maybe, 50 not relevant
(26 no platform-level boarding/alighting, 13 BRT planning or
operations only, 10 other meaning of BRT, 1 other). v0.3 is frozen as
the final search string, with no BRT terms added.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/progress/SLR/brt_missed_sample.xlsx
+++ b/progress/SLR/brt_missed_sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git2026\research-progress\progress\SLR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBB0028A-EB8B-4E88-B1BC-73C66066D876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8ACDBC8-AEC9-4A94-A30D-31987D4C5AEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="22150" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-200" yWindow="0" windowWidth="22930" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sample" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="257">
   <si>
     <t>sample_id</t>
   </si>
@@ -1188,7 +1188,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="319" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="348" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="I5" s="3"/>
     </row>
-    <row r="6" spans="1:9" ht="203" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>29</v>
       </c>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I6" s="3"/>
     </row>
-    <row r="7" spans="1:9" ht="232" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="261" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>34</v>
       </c>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="174" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>39</v>
       </c>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="I8" s="3"/>
     </row>
-    <row r="9" spans="1:9" ht="174" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>44</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="246.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>49</v>
       </c>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="I10" s="3"/>
     </row>
-    <row r="11" spans="1:9" ht="203" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>54</v>
       </c>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="I11" s="3"/>
     </row>
-    <row r="12" spans="1:9" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>59</v>
       </c>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="I29" s="3"/>
     </row>
-    <row r="30" spans="1:9" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" ht="290" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>142</v>
       </c>
@@ -1959,11 +1959,15 @@
       <c r="F30" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
+      <c r="G30" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="I30" s="3"/>
     </row>
-    <row r="31" spans="1:9" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>147</v>
       </c>
@@ -1982,11 +1986,15 @@
       <c r="F31" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
+      <c r="G31" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="I31" s="3"/>
     </row>
-    <row r="32" spans="1:9" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" ht="232" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>152</v>
       </c>
@@ -2005,11 +2013,15 @@
       <c r="F32" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
+      <c r="G32" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>253</v>
+      </c>
       <c r="I32" s="3"/>
     </row>
-    <row r="33" spans="1:9" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" ht="145" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>157</v>
       </c>
@@ -2026,11 +2038,15 @@
       <c r="F33" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
+      <c r="G33" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>253</v>
+      </c>
       <c r="I33" s="3"/>
     </row>
-    <row r="34" spans="1:9" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" ht="232" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>161</v>
       </c>
@@ -2049,11 +2065,15 @@
       <c r="F34" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
+      <c r="G34" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="I34" s="3"/>
     </row>
-    <row r="35" spans="1:9" ht="304.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
         <v>166</v>
       </c>
@@ -2072,11 +2092,15 @@
       <c r="F35" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
+      <c r="G35" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="I35" s="3"/>
     </row>
-    <row r="36" spans="1:9" ht="203" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" ht="232" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>171</v>
       </c>
@@ -2095,11 +2119,15 @@
       <c r="F36" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
+      <c r="G36" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="I36" s="3"/>
     </row>
-    <row r="37" spans="1:9" ht="203" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>176</v>
       </c>
@@ -2118,11 +2146,15 @@
       <c r="F37" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
+      <c r="G37" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="I37" s="3"/>
     </row>
-    <row r="38" spans="1:9" ht="246.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" ht="261" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>181</v>
       </c>
@@ -2141,8 +2173,12 @@
       <c r="F38" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
+      <c r="G38" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="I38" s="3"/>
     </row>
     <row r="39" spans="1:9" ht="87" x14ac:dyDescent="0.35">
@@ -2164,11 +2200,15 @@
       <c r="F39" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
+      <c r="G39" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="I39" s="3"/>
     </row>
-    <row r="40" spans="1:9" ht="174" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>191</v>
       </c>
@@ -2187,11 +2227,15 @@
       <c r="F40" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="G40" s="3"/>
-      <c r="H40" s="3"/>
+      <c r="G40" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="I40" s="3"/>
     </row>
-    <row r="41" spans="1:9" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" ht="174" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
         <v>196</v>
       </c>
@@ -2210,11 +2254,15 @@
       <c r="F41" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="G41" s="3"/>
-      <c r="H41" s="3"/>
+      <c r="G41" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>253</v>
+      </c>
       <c r="I41" s="3"/>
     </row>
-    <row r="42" spans="1:9" ht="174" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>201</v>
       </c>
@@ -2233,11 +2281,15 @@
       <c r="F42" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
+      <c r="G42" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="I42" s="3"/>
     </row>
-    <row r="43" spans="1:9" ht="246.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>206</v>
       </c>
@@ -2256,11 +2308,15 @@
       <c r="F43" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="G43" s="3"/>
-      <c r="H43" s="3"/>
+      <c r="G43" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="I43" s="3"/>
     </row>
-    <row r="44" spans="1:9" ht="174" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" ht="203" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
         <v>211</v>
       </c>
@@ -2279,11 +2335,15 @@
       <c r="F44" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="G44" s="3"/>
-      <c r="H44" s="3"/>
+      <c r="G44" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>253</v>
+      </c>
       <c r="I44" s="3"/>
     </row>
-    <row r="45" spans="1:9" ht="290" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
         <v>216</v>
       </c>
@@ -2302,11 +2362,15 @@
       <c r="F45" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="G45" s="3"/>
-      <c r="H45" s="3"/>
+      <c r="G45" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="I45" s="3"/>
     </row>
-    <row r="46" spans="1:9" ht="391.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>221</v>
       </c>
@@ -2325,11 +2389,15 @@
       <c r="F46" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
+      <c r="G46" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>253</v>
+      </c>
       <c r="I46" s="3"/>
     </row>
-    <row r="47" spans="1:9" ht="203" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
         <v>226</v>
       </c>
@@ -2348,11 +2416,15 @@
       <c r="F47" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
+      <c r="G47" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>253</v>
+      </c>
       <c r="I47" s="3"/>
     </row>
-    <row r="48" spans="1:9" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" ht="203" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
         <v>231</v>
       </c>
@@ -2371,8 +2443,12 @@
       <c r="F48" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="G48" s="3"/>
-      <c r="H48" s="3"/>
+      <c r="G48" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>253</v>
+      </c>
       <c r="I48" s="3"/>
     </row>
     <row r="49" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
@@ -2394,11 +2470,15 @@
       <c r="F49" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="G49" s="3"/>
-      <c r="H49" s="3"/>
+      <c r="G49" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="I49" s="3"/>
     </row>
-    <row r="50" spans="1:9" ht="290" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:9" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
         <v>241</v>
       </c>
@@ -2417,11 +2497,15 @@
       <c r="F50" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="G50" s="3"/>
-      <c r="H50" s="3"/>
+      <c r="G50" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>254</v>
+      </c>
       <c r="I50" s="3"/>
     </row>
-    <row r="51" spans="1:9" ht="391.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>246</v>
       </c>
@@ -2440,8 +2524,12 @@
       <c r="F51" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="G51" s="3"/>
-      <c r="H51" s="3"/>
+      <c r="G51" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>253</v>
+      </c>
       <c r="I51" s="3"/>
     </row>
   </sheetData>

</xml_diff>